<commit_message>
Search the text of PDF printouts; list future features
When an attached PDF is inserted as a printout, each page's text layer is
kept with its picture. Search lists those pages under In printouts, page
search counts the matches and outlines the picture, and page.html lays the
text transparently over each printout. Plain attachments are never searched
by content. Search index version 4 rebuilds on first open.

docs/dev/FUTURE_FEATURES.md lists the follow-ups and the gaps noted in the
feature comparison, for later consideration.
</commit_message>
<xml_diff>
--- a/docs/PageBinder-feature-comparison.xlsx
+++ b/docs/PageBinder-feature-comparison.xlsx
@@ -877,7 +877,7 @@
     <t xml:space="preserve">Searches inside attachments</t>
   </si>
   <si>
-    <t xml:space="preserve">Partial: text of saved emails</t>
+    <t xml:space="preserve">Partial: saved emails and PDF printouts (not plain attachments)</t>
   </si>
   <si>
     <t xml:space="preserve">Yes: OCR of images and PDFs *</t>
@@ -6391,7 +6391,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="19" t="s">
         <v>282</v>
       </c>

</xml_diff>